<commit_message>
Incorporate historical reserve margin instead of target.
</commit_message>
<xml_diff>
--- a/InputData/elec/RM/Reserve Margin.xlsx
+++ b/InputData/elec/RM/Reserve Margin.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\South Korea\Models\eps-southkorea\InputData\elec\RM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{279CE630-958D-4440-8649-55CFAD946665}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE6A24FB-393B-4AC1-A90E-BB6EC91807A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="23520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
-    <sheet name="RM" sheetId="2" r:id="rId2"/>
+    <sheet name="Historical" sheetId="3" r:id="rId2"/>
+    <sheet name="RM" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="41">
   <si>
     <t>RM Reserve Margin</t>
   </si>
@@ -67,13 +68,110 @@
   </si>
   <si>
     <t>https://www.iea.org/articles/korea-electricity-security-policy</t>
+  </si>
+  <si>
+    <t>Target</t>
+  </si>
+  <si>
+    <t>Historical</t>
+  </si>
+  <si>
+    <t>Korea Power Exchange</t>
+  </si>
+  <si>
+    <t>EPSIS</t>
+  </si>
+  <si>
+    <t>https://epsis.kpx.or.kr/epsisnew/selectEkgeEpsMepChart.do?menuId=030100&amp;locale=eng</t>
+  </si>
+  <si>
+    <t>Peak/Base Demand</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Month</t>
+  </si>
+  <si>
+    <t>Day</t>
+  </si>
+  <si>
+    <t>Installed
+Capacity (MW)</t>
+  </si>
+  <si>
+    <t>Available
+Capacity (MW)</t>
+  </si>
+  <si>
+    <t>Peak
+Demand (MW)</t>
+  </si>
+  <si>
+    <t>Base
+Demand (MW)</t>
+  </si>
+  <si>
+    <t>Reserve (MW)</t>
+  </si>
+  <si>
+    <t>Reserve
+Margin (%)</t>
+  </si>
+  <si>
+    <t>Peak
+Demand Date</t>
+  </si>
+  <si>
+    <t>Base
+Demand Date</t>
+  </si>
+  <si>
+    <t>08</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>2025/08/25(18:00)</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>2024/08/20(17:00)</t>
+  </si>
+  <si>
+    <t>07</t>
+  </si>
+  <si>
+    <t>2023/08/07(17:00)</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>2022/12/23(11:00)</t>
+  </si>
+  <si>
+    <t>27</t>
+  </si>
+  <si>
+    <t>2021/07/27(18:00)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -89,16 +187,46 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="13"/>
+      <color rgb="FF000000"/>
+      <name val="맑은 고딕"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF333333"/>
+      <name val="맑은 고딕"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF31393F"/>
+      <name val="맑은 고딕"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDDDDD"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -106,19 +234,78 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF999999"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFEAEAEA"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFEAEAEA"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFDDDDDD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFDDDDDD"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{BFCEC036-89F3-4B56-8BDD-8AF117EE44CA}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -420,54 +607,95 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E19"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="B4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B4" s="2">
+    <row r="5" spans="1:5">
+      <c r="B5" s="2">
         <v>2025</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B5" s="2" t="s">
+    <row r="6" spans="1:5">
+      <c r="B6" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B6" t="s">
+    <row r="7" spans="1:5">
+      <c r="B7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+    <row r="9" spans="1:5">
+      <c r="B9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="B10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="B11" s="2">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="B12" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="B13" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="B14" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="17" spans="1:1">
+      <c r="A17" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="18" spans="1:1">
+      <c r="A18" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="19" spans="1:1">
+      <c r="A19" t="s">
         <v>6</v>
       </c>
     </row>
@@ -478,180 +706,387 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E85C82EA-7685-401D-8FEC-A2098B525E60}">
+  <dimension ref="A1:K6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:11" ht="40.5">
+      <c r="A1" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" s="9">
+        <v>2025</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D2" s="7">
+        <v>155385</v>
+      </c>
+      <c r="E2" s="7">
+        <v>105011</v>
+      </c>
+      <c r="F2" s="7">
+        <v>95951</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="H2" s="7">
+        <v>9060</v>
+      </c>
+      <c r="I2" s="7">
+        <v>9.4</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" s="9">
+        <v>2024</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" s="7">
+        <v>149179</v>
+      </c>
+      <c r="E3" s="7">
+        <v>105360</v>
+      </c>
+      <c r="F3" s="7">
+        <v>97115</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="H3" s="7">
+        <v>8245</v>
+      </c>
+      <c r="I3" s="7">
+        <v>8.5</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="K3" s="8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" s="9">
+        <v>2023</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D4" s="7">
+        <v>142567</v>
+      </c>
+      <c r="E4" s="7">
+        <v>104297</v>
+      </c>
+      <c r="F4" s="7">
+        <v>93615</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="H4" s="7">
+        <v>10682</v>
+      </c>
+      <c r="I4" s="7">
+        <v>11.4</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" s="9">
+        <v>2022</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" s="7">
+        <v>137938</v>
+      </c>
+      <c r="E5" s="7">
+        <v>105628</v>
+      </c>
+      <c r="F5" s="7">
+        <v>94509</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="H5" s="7">
+        <v>11119</v>
+      </c>
+      <c r="I5" s="7">
+        <v>11.8</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="K5" s="8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" s="9">
+        <v>2021</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6" s="7">
+        <v>131330</v>
+      </c>
+      <c r="E6" s="7">
+        <v>100739</v>
+      </c>
+      <c r="F6" s="7">
+        <v>91141</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="H6" s="7">
+        <v>9598</v>
+      </c>
+      <c r="I6" s="7">
+        <v>10.5</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="K6" s="8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
-  <dimension ref="A1:AK2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AE2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31">
       <c r="A1" t="s">
         <v>7</v>
       </c>
       <c r="B1">
-        <v>2015</v>
+        <v>2021</v>
       </c>
       <c r="C1">
-        <v>2016</v>
+        <v>2022</v>
       </c>
       <c r="D1">
-        <v>2017</v>
+        <v>2023</v>
       </c>
       <c r="E1">
-        <v>2018</v>
+        <v>2024</v>
       </c>
       <c r="F1">
-        <v>2019</v>
-      </c>
-      <c r="G1">
-        <v>2020</v>
+        <v>2025</v>
+      </c>
+      <c r="G1" s="10">
+        <v>2026</v>
       </c>
       <c r="H1">
-        <v>2021</v>
+        <v>2027</v>
       </c>
       <c r="I1">
-        <v>2022</v>
+        <v>2028</v>
       </c>
       <c r="J1">
-        <v>2023</v>
+        <v>2029</v>
       </c>
       <c r="K1">
-        <v>2024</v>
+        <v>2030</v>
       </c>
       <c r="L1">
-        <v>2025</v>
+        <v>2031</v>
       </c>
       <c r="M1">
-        <v>2026</v>
+        <v>2032</v>
       </c>
       <c r="N1">
-        <v>2027</v>
+        <v>2033</v>
       </c>
       <c r="O1">
-        <v>2028</v>
+        <v>2034</v>
       </c>
       <c r="P1">
-        <v>2029</v>
+        <v>2035</v>
       </c>
       <c r="Q1">
-        <v>2030</v>
+        <v>2036</v>
       </c>
       <c r="R1">
-        <v>2031</v>
+        <v>2037</v>
       </c>
       <c r="S1">
-        <v>2032</v>
+        <v>2038</v>
       </c>
       <c r="T1">
-        <v>2033</v>
+        <v>2039</v>
       </c>
       <c r="U1">
-        <v>2034</v>
+        <v>2040</v>
       </c>
       <c r="V1">
-        <v>2035</v>
+        <v>2041</v>
       </c>
       <c r="W1">
-        <v>2036</v>
+        <v>2042</v>
       </c>
       <c r="X1">
-        <v>2037</v>
+        <v>2043</v>
       </c>
       <c r="Y1">
-        <v>2038</v>
+        <v>2044</v>
       </c>
       <c r="Z1">
-        <v>2039</v>
+        <v>2045</v>
       </c>
       <c r="AA1">
-        <v>2040</v>
+        <v>2046</v>
       </c>
       <c r="AB1">
-        <v>2041</v>
+        <v>2047</v>
       </c>
       <c r="AC1">
-        <v>2042</v>
+        <v>2048</v>
       </c>
       <c r="AD1">
-        <v>2043</v>
+        <v>2049</v>
       </c>
       <c r="AE1">
-        <v>2044</v>
-      </c>
-      <c r="AF1">
-        <v>2045</v>
-      </c>
-      <c r="AG1">
-        <v>2046</v>
-      </c>
-      <c r="AH1">
-        <v>2047</v>
-      </c>
-      <c r="AI1">
-        <v>2048</v>
-      </c>
-      <c r="AJ1">
-        <v>2049</v>
-      </c>
-      <c r="AK1">
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2">
+        <f>INDEX(Historical!$I$2:$I$60,MATCH(RM!B1,Historical!$A$2:$A$6,0),1)/100</f>
+        <v>0.105</v>
+      </c>
+      <c r="C2">
+        <f>INDEX(Historical!$I$2:$I$60,MATCH(RM!C1,Historical!$A$2:$A$6,0),1)/100</f>
+        <v>0.11800000000000001</v>
+      </c>
+      <c r="D2">
+        <f>INDEX(Historical!$I$2:$I$60,MATCH(RM!D1,Historical!$A$2:$A$6,0),1)/100</f>
+        <v>0.114</v>
+      </c>
+      <c r="E2">
+        <f>INDEX(Historical!$I$2:$I$60,MATCH(RM!E1,Historical!$A$2:$A$6,0),1)/100</f>
+        <v>8.5000000000000006E-2</v>
+      </c>
+      <c r="F2">
+        <f>INDEX(Historical!$I$2:$I$60,MATCH(RM!F1,Historical!$A$2:$A$6,0),1)/100</f>
+        <v>9.4E-2</v>
+      </c>
+      <c r="G2" s="10">
         <v>0.2</v>
       </c>
-      <c r="C2">
-        <v>0.2</v>
-      </c>
-      <c r="D2">
-        <v>0.2</v>
-      </c>
-      <c r="E2">
-        <v>0.2</v>
-      </c>
-      <c r="F2">
-        <v>0.2</v>
-      </c>
-      <c r="G2">
-        <v>0.2</v>
-      </c>
       <c r="H2">
-        <v>0.2</v>
+        <v>0.21</v>
       </c>
       <c r="I2">
-        <v>0.2</v>
+        <v>0.21</v>
       </c>
       <c r="J2">
-        <v>0.2</v>
+        <v>0.21</v>
       </c>
       <c r="K2">
-        <v>0.2</v>
+        <v>0.21</v>
       </c>
       <c r="L2">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="M2">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="N2">
-        <v>0.21</v>
+        <v>0.22</v>
       </c>
       <c r="O2">
-        <v>0.21</v>
+        <v>0.22</v>
       </c>
       <c r="P2">
-        <v>0.21</v>
+        <v>0.22</v>
       </c>
       <c r="Q2">
-        <v>0.21</v>
+        <v>0.22</v>
       </c>
       <c r="R2">
         <v>0.22</v>
@@ -693,24 +1128,6 @@
         <v>0.22</v>
       </c>
       <c r="AE2">
-        <v>0.22</v>
-      </c>
-      <c r="AF2">
-        <v>0.22</v>
-      </c>
-      <c r="AG2">
-        <v>0.22</v>
-      </c>
-      <c r="AH2">
-        <v>0.22</v>
-      </c>
-      <c r="AI2">
-        <v>0.22</v>
-      </c>
-      <c r="AJ2">
-        <v>0.22</v>
-      </c>
-      <c r="AK2">
         <v>0.22</v>
       </c>
     </row>
@@ -864,18 +1281,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -897,18 +1314,18 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B0BE9E85-1A0B-4D4C-BDAA-A91DCB3B1348}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AD3D1029-3329-4E1F-A846-3AAC857EA878}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B0BE9E85-1A0B-4D4C-BDAA-A91DCB3B1348}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>